<commit_message>
updated new manual deployment
</commit_message>
<xml_diff>
--- a/docs/notes/Overall GCP List.xlsx
+++ b/docs/notes/Overall GCP List.xlsx
@@ -5165,14 +5165,15 @@
   <cols>
     <col min="1" max="1" width="7.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="33.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.88671875" hidden="1" customWidth="1"/>
     <col min="4" max="4" width="10.109375" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="8.6640625" hidden="1" customWidth="1"/>
     <col min="6" max="6" width="71.6640625" hidden="1" customWidth="1"/>
     <col min="7" max="7" width="22.44140625" hidden="1" customWidth="1"/>
     <col min="8" max="8" width="9.6640625" hidden="1" customWidth="1"/>
     <col min="9" max="9" width="10.109375" hidden="1" customWidth="1"/>
-    <col min="10" max="10" width="0" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="71" hidden="1" customWidth="1"/>
+    <col min="11" max="11" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">

</xml_diff>